<commit_message>
map logical numbering to match physical and software
</commit_message>
<xml_diff>
--- a/mappings.xlsx
+++ b/mappings.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="V:\_Working\BreezeWorks\GagWriter Remastered\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3360BB67-2782-4874-9CD4-301831A4BC04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09C252B9-C23B-4586-A64D-A6BABCCFCD9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13755" yWindow="285" windowWidth="29490" windowHeight="30945" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="57495" yWindow="8025" windowWidth="19905" windowHeight="16305" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="128">
   <si>
     <t>Central</t>
   </si>
@@ -378,6 +378,48 @@
   </si>
   <si>
     <t>1,</t>
+  </si>
+  <si>
+    <t>simultaneous image/sound</t>
+  </si>
+  <si>
+    <t>5,</t>
+  </si>
+  <si>
+    <t>gpio expander</t>
+  </si>
+  <si>
+    <t>A7</t>
+  </si>
+  <si>
+    <t>A3</t>
+  </si>
+  <si>
+    <t>A1</t>
+  </si>
+  <si>
+    <t>A4</t>
+  </si>
+  <si>
+    <t>A6</t>
+  </si>
+  <si>
+    <t>A0</t>
+  </si>
+  <si>
+    <t>A2</t>
+  </si>
+  <si>
+    <t>A5</t>
+  </si>
+  <si>
+    <t>sig reserved</t>
+  </si>
+  <si>
+    <t>B0</t>
+  </si>
+  <si>
+    <t>0,6 I guess</t>
   </si>
 </sst>
 </file>
@@ -775,7 +817,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B4:AP73"/>
+  <dimension ref="B4:AP76"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="11" customWidth="1"/>
@@ -3130,7 +3172,10 @@
         <v>14</v>
       </c>
       <c r="F29" t="s">
-        <v>55</v>
+        <v>114</v>
+      </c>
+      <c r="G29" t="s">
+        <v>115</v>
       </c>
       <c r="J29" t="s">
         <v>35</v>
@@ -3233,10 +3278,7 @@
         <v>12</v>
       </c>
       <c r="F30" t="s">
-        <v>56</v>
-      </c>
-      <c r="G30">
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="J30" t="s">
         <v>93</v>
@@ -3339,10 +3381,10 @@
         <v>44</v>
       </c>
       <c r="F31" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G31">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J31" t="s">
         <v>94</v>
@@ -3448,10 +3490,10 @@
         <v>31</v>
       </c>
       <c r="F32" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G32">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J32" t="s">
         <v>74</v>
@@ -3554,10 +3596,10 @@
         <v>41</v>
       </c>
       <c r="F33" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="G33">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J33" t="s">
         <v>15</v>
@@ -3663,10 +3705,10 @@
         <v>21</v>
       </c>
       <c r="F34" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G34">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J34" t="s">
         <v>5</v>
@@ -3769,10 +3811,10 @@
         <v>23</v>
       </c>
       <c r="F35" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G35">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J35" t="s">
         <v>33</v>
@@ -3875,10 +3917,10 @@
         <v>24</v>
       </c>
       <c r="F36" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G36">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J36" t="s">
         <v>25</v>
@@ -3981,7 +4023,10 @@
         <v>32</v>
       </c>
       <c r="F37" t="s">
-        <v>63</v>
+        <v>62</v>
+      </c>
+      <c r="G37">
+        <v>6</v>
       </c>
       <c r="J37" t="s">
         <v>19</v>
@@ -4087,10 +4132,7 @@
         <v>10</v>
       </c>
       <c r="F38" t="s">
-        <v>64</v>
-      </c>
-      <c r="G38">
-        <v>0</v>
+        <v>63</v>
       </c>
       <c r="S38">
         <v>4</v>
@@ -4187,13 +4229,16 @@
         <v>34</v>
       </c>
       <c r="F39" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G39">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J39" t="s">
         <v>95</v>
+      </c>
+      <c r="K39" t="s">
+        <v>127</v>
       </c>
       <c r="S39">
         <v>4</v>
@@ -4293,10 +4338,10 @@
         <v>42</v>
       </c>
       <c r="F40" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G40">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J40">
         <v>1</v>
@@ -4396,10 +4441,10 @@
         <v>43</v>
       </c>
       <c r="F41" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G41">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J41">
         <v>2</v>
@@ -4499,10 +4544,10 @@
         <v>111</v>
       </c>
       <c r="F42" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G42">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J42">
         <v>3</v>
@@ -4602,10 +4647,10 @@
         <v>109</v>
       </c>
       <c r="F43" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G43">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J43">
         <v>4</v>
@@ -4705,10 +4750,10 @@
         <v>107</v>
       </c>
       <c r="F44" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G44">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J44">
         <v>5</v>
@@ -4806,6 +4851,12 @@
       </c>
       <c r="D45" s="1">
         <v>15</v>
+      </c>
+      <c r="F45" t="s">
+        <v>70</v>
+      </c>
+      <c r="G45">
+        <v>6</v>
       </c>
       <c r="S45">
         <v>5</v>
@@ -5853,8 +5904,11 @@
       <c r="O64" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="65" spans="11:15" x14ac:dyDescent="0.25">
+      <c r="Q64" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="65" spans="11:17" x14ac:dyDescent="0.25">
       <c r="K65" t="s">
         <v>83</v>
       </c>
@@ -5867,8 +5921,11 @@
       <c r="O65" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="66" spans="11:15" x14ac:dyDescent="0.25">
+      <c r="Q65" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="66" spans="11:17" x14ac:dyDescent="0.25">
       <c r="K66" t="s">
         <v>84</v>
       </c>
@@ -5881,8 +5938,11 @@
       <c r="O66" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="67" spans="11:15" x14ac:dyDescent="0.25">
+      <c r="Q66" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="67" spans="11:17" x14ac:dyDescent="0.25">
       <c r="K67" t="s">
         <v>85</v>
       </c>
@@ -5895,8 +5955,11 @@
       <c r="O67" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="68" spans="11:15" x14ac:dyDescent="0.25">
+      <c r="Q67" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="68" spans="11:17" x14ac:dyDescent="0.25">
       <c r="K68" t="s">
         <v>86</v>
       </c>
@@ -5909,8 +5972,11 @@
       <c r="O68" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="69" spans="11:15" x14ac:dyDescent="0.25">
+      <c r="Q68" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="69" spans="11:17" x14ac:dyDescent="0.25">
       <c r="K69" t="s">
         <v>87</v>
       </c>
@@ -5923,8 +5989,11 @@
       <c r="O69" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="70" spans="11:15" x14ac:dyDescent="0.25">
+      <c r="Q69" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="70" spans="11:17" x14ac:dyDescent="0.25">
       <c r="K70" t="s">
         <v>88</v>
       </c>
@@ -5937,8 +6006,11 @@
       <c r="O70" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="71" spans="11:15" x14ac:dyDescent="0.25">
+      <c r="Q70" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="71" spans="11:17" x14ac:dyDescent="0.25">
       <c r="K71" t="s">
         <v>89</v>
       </c>
@@ -5951,13 +6023,27 @@
       <c r="O71" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="73" spans="11:15" x14ac:dyDescent="0.25">
+      <c r="Q71" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="73" spans="11:17" x14ac:dyDescent="0.25">
       <c r="K73" t="s">
         <v>96</v>
       </c>
       <c r="O73" t="s">
         <v>25</v>
+      </c>
+      <c r="Q73" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="76" spans="11:17" x14ac:dyDescent="0.25">
+      <c r="K76" t="s">
+        <v>125</v>
+      </c>
+      <c r="Q76" t="s">
+        <v>126</v>
       </c>
     </row>
   </sheetData>

</xml_diff>